<commit_message>
Ocarina of Time Remake for Nintendo Switch 2
</commit_message>
<xml_diff>
--- a/ZELDA.xlsx
+++ b/ZELDA.xlsx
@@ -8,22 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1358A9F-6CAA-4001-82FD-6909EF5CB4F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB5AA8B-AA15-48EC-A67F-49733D5729A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{544A5710-79AF-4C5F-8C3A-ADA1AE421E72}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{544A5710-79AF-4C5F-8C3A-ADA1AE421E72}"/>
   </bookViews>
   <sheets>
     <sheet name="ZELDA" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ZELDA!$A$1:$L$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ZELDA!$A$1:$L$37</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="164">
   <si>
     <t>id</t>
   </si>
@@ -506,6 +506,15 @@
   </si>
   <si>
     <t>https://images.igdb.com/igdb/image/upload/t_cover_big_2x/cob9n1.webp</t>
+  </si>
+  <si>
+    <t>zd36</t>
+  </si>
+  <si>
+    <t>https://images.igdb.com/igdb/image/upload/t_cover_big_2x/cocv5r.webp</t>
+  </si>
+  <si>
+    <t>https://www.igdb.com/games/the-legend-of-zelda-ocarina-of-time--1</t>
   </si>
 </sst>
 </file>
@@ -1383,16 +1392,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D7D8C5C-82D0-4767-86A0-EC7D017C2964}">
-  <dimension ref="A1:M36"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:M37"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="4" max="4" width="46.85546875" customWidth="1"/>
-    <col min="9" max="9" width="27.28515625" customWidth="1"/>
-    <col min="10" max="10" width="49.140625" customWidth="1"/>
-    <col min="11" max="11" width="72.85546875" customWidth="1"/>
+    <col min="4" max="4" width="46.86328125" customWidth="1"/>
+    <col min="9" max="9" width="27.265625" customWidth="1"/>
+    <col min="10" max="10" width="49.1328125" customWidth="1"/>
+    <col min="11" max="11" width="72.86328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1433,111 +1442,111 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B2">
+        <v>20</v>
+      </c>
+      <c r="C2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>27</v>
-      </c>
       <c r="D2" t="s">
-        <v>52</v>
+        <v>13</v>
       </c>
       <c r="I2" t="s">
         <v>14</v>
       </c>
       <c r="J2" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="K2" t="s">
-        <v>126</v>
+        <v>145</v>
       </c>
       <c r="M2" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>86</v>
       </c>
       <c r="B3">
+        <v>32</v>
+      </c>
+      <c r="C3">
         <v>2</v>
       </c>
-      <c r="C3">
-        <v>28</v>
-      </c>
       <c r="D3" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="I3" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="J3" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="K3" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
       <c r="M3" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="B4">
+        <v>13</v>
+      </c>
+      <c r="C4">
         <v>3</v>
       </c>
-      <c r="C4">
-        <v>9</v>
-      </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="I4" t="s">
         <v>14</v>
       </c>
       <c r="J4" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="K4" t="s">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="M4" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="B5">
+        <v>10</v>
+      </c>
+      <c r="C5">
         <v>4</v>
       </c>
-      <c r="C5">
+      <c r="D5" t="s">
         <v>19</v>
       </c>
-      <c r="D5" t="s">
-        <v>40</v>
-      </c>
       <c r="I5" t="s">
         <v>14</v>
       </c>
       <c r="J5" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="K5" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="M5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1563,137 +1572,137 @@
         <v>98</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>60</v>
       </c>
       <c r="B7">
+        <v>19</v>
+      </c>
+      <c r="C7">
         <v>6</v>
       </c>
-      <c r="C7">
-        <v>20</v>
-      </c>
       <c r="D7" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="I7" t="s">
         <v>65</v>
       </c>
       <c r="J7" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="K7" t="s">
-        <v>131</v>
+        <v>144</v>
       </c>
       <c r="M7" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>161</v>
       </c>
       <c r="B8">
-        <v>7</v>
+        <v>36</v>
       </c>
       <c r="C8">
         <v>7</v>
       </c>
       <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" t="s">
+        <v>65</v>
+      </c>
+      <c r="J8" t="s">
+        <v>15</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="M8" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
         <v>23</v>
       </c>
-      <c r="I8" t="s">
-        <v>14</v>
-      </c>
-      <c r="J8" t="s">
+      <c r="I9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" t="s">
         <v>24</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K9" t="s">
         <v>132</v>
       </c>
-      <c r="M8" t="s">
+      <c r="M9" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>32</v>
-      </c>
-      <c r="B9">
-        <v>8</v>
-      </c>
-      <c r="C9">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s">
-        <v>31</v>
-      </c>
-      <c r="I9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J9" t="s">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10">
+        <v>24</v>
+      </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
+      <c r="D10" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" t="s">
+        <v>65</v>
+      </c>
+      <c r="J10" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" t="s">
+        <v>149</v>
+      </c>
+      <c r="M10" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="C11">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" t="s">
         <v>27</v>
       </c>
-      <c r="K9" t="s">
-        <v>133</v>
-      </c>
-      <c r="M9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10">
-        <v>9</v>
-      </c>
-      <c r="C10">
-        <v>13</v>
-      </c>
-      <c r="D10" t="s">
-        <v>33</v>
-      </c>
-      <c r="I10" t="s">
-        <v>14</v>
-      </c>
-      <c r="J10" t="s">
-        <v>27</v>
-      </c>
-      <c r="K10" t="s">
-        <v>134</v>
-      </c>
-      <c r="M10" t="s">
+      <c r="K11" t="s">
+        <v>128</v>
+      </c>
+      <c r="M11" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11">
-        <v>10</v>
-      </c>
-      <c r="C11">
-        <v>4</v>
-      </c>
-      <c r="D11" t="s">
-        <v>19</v>
-      </c>
-      <c r="I11" t="s">
-        <v>14</v>
-      </c>
-      <c r="J11" t="s">
-        <v>15</v>
-      </c>
-      <c r="K11" t="s">
-        <v>135</v>
-      </c>
-      <c r="M11" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>47</v>
       </c>
@@ -1701,7 +1710,7 @@
         <v>11</v>
       </c>
       <c r="C12">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D12" t="s">
         <v>29</v>
@@ -1716,140 +1725,140 @@
         <v>136</v>
       </c>
       <c r="M12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13">
+        <v>21</v>
+      </c>
+      <c r="C13">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s">
+        <v>70</v>
+      </c>
+      <c r="I13" t="s">
+        <v>65</v>
+      </c>
+      <c r="J13" t="s">
+        <v>36</v>
+      </c>
+      <c r="K13" t="s">
+        <v>146</v>
+      </c>
+      <c r="M13" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14">
+        <v>8</v>
+      </c>
+      <c r="C14">
+        <v>13</v>
+      </c>
+      <c r="D14" t="s">
+        <v>31</v>
+      </c>
+      <c r="I14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" t="s">
+        <v>27</v>
+      </c>
+      <c r="K14" t="s">
+        <v>133</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15">
+        <v>9</v>
+      </c>
+      <c r="C15">
+        <v>14</v>
+      </c>
+      <c r="D15" t="s">
+        <v>33</v>
+      </c>
+      <c r="I15" t="s">
+        <v>14</v>
+      </c>
+      <c r="J15" t="s">
+        <v>27</v>
+      </c>
+      <c r="K15" t="s">
+        <v>134</v>
+      </c>
+      <c r="M15" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16">
         <v>16</v>
       </c>
-      <c r="B13">
-        <v>12</v>
-      </c>
-      <c r="C13">
-        <v>25</v>
-      </c>
-      <c r="D13" t="s">
-        <v>48</v>
-      </c>
-      <c r="I13" t="s">
-        <v>14</v>
-      </c>
-      <c r="J13" t="s">
+      <c r="C16">
+        <v>15</v>
+      </c>
+      <c r="D16" t="s">
+        <v>35</v>
+      </c>
+      <c r="I16" t="s">
+        <v>14</v>
+      </c>
+      <c r="J16" t="s">
+        <v>36</v>
+      </c>
+      <c r="K16" t="s">
+        <v>141</v>
+      </c>
+      <c r="M16" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>34</v>
+      </c>
+      <c r="B17">
+        <v>14</v>
+      </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
+      <c r="D17" t="s">
+        <v>66</v>
+      </c>
+      <c r="I17" t="s">
+        <v>67</v>
+      </c>
+      <c r="J17" t="s">
         <v>24</v>
       </c>
-      <c r="K13" t="s">
-        <v>137</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14">
-        <v>13</v>
-      </c>
-      <c r="C14">
-        <v>3</v>
-      </c>
-      <c r="D14" t="s">
-        <v>17</v>
-      </c>
-      <c r="I14" t="s">
-        <v>14</v>
-      </c>
-      <c r="J14" t="s">
-        <v>15</v>
-      </c>
-      <c r="K14" t="s">
-        <v>138</v>
-      </c>
-      <c r="M14" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>34</v>
-      </c>
-      <c r="B15">
-        <v>14</v>
-      </c>
-      <c r="C15">
-        <v>15</v>
-      </c>
-      <c r="D15" t="s">
-        <v>66</v>
-      </c>
-      <c r="I15" t="s">
-        <v>67</v>
-      </c>
-      <c r="J15" t="s">
-        <v>24</v>
-      </c>
-      <c r="K15" t="s">
+      <c r="K17" t="s">
         <v>139</v>
       </c>
-      <c r="M15" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>49</v>
-      </c>
-      <c r="B16">
-        <v>15</v>
-      </c>
-      <c r="C16">
-        <v>17</v>
-      </c>
-      <c r="D16" t="s">
-        <v>38</v>
-      </c>
-      <c r="I16" t="s">
-        <v>14</v>
-      </c>
-      <c r="J16" t="s">
-        <v>24</v>
-      </c>
-      <c r="K16" t="s">
-        <v>140</v>
-      </c>
-      <c r="M16" t="s">
+      <c r="M17" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>12</v>
-      </c>
-      <c r="B17">
-        <v>16</v>
-      </c>
-      <c r="C17">
-        <v>14</v>
-      </c>
-      <c r="D17" t="s">
-        <v>35</v>
-      </c>
-      <c r="I17" t="s">
-        <v>14</v>
-      </c>
-      <c r="J17" t="s">
-        <v>36</v>
-      </c>
-      <c r="K17" t="s">
-        <v>141</v>
-      </c>
-      <c r="M17" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -1857,7 +1866,7 @@
         <v>17</v>
       </c>
       <c r="C18">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D18" t="s">
         <v>68</v>
@@ -1872,203 +1881,203 @@
         <v>142</v>
       </c>
       <c r="M18" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>49</v>
+      </c>
+      <c r="B19">
+        <v>15</v>
+      </c>
+      <c r="C19">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>38</v>
+      </c>
+      <c r="I19" t="s">
+        <v>14</v>
+      </c>
+      <c r="J19" t="s">
+        <v>24</v>
+      </c>
+      <c r="K19" t="s">
+        <v>140</v>
+      </c>
+      <c r="M19" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>45</v>
-      </c>
-      <c r="B19">
-        <v>18</v>
-      </c>
-      <c r="C19">
-        <v>26</v>
-      </c>
-      <c r="D19" t="s">
-        <v>50</v>
-      </c>
-      <c r="I19" t="s">
-        <v>14</v>
-      </c>
-      <c r="J19" t="s">
-        <v>36</v>
-      </c>
-      <c r="K19" t="s">
-        <v>143</v>
-      </c>
-      <c r="M19" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="B20">
+        <v>27</v>
+      </c>
+      <c r="C20">
         <v>19</v>
       </c>
-      <c r="C20">
-        <v>6</v>
-      </c>
       <c r="D20" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="I20" t="s">
         <v>65</v>
       </c>
       <c r="J20" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="K20" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="M20" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21">
+        <v>4</v>
+      </c>
+      <c r="C21">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>40</v>
+      </c>
+      <c r="I21" t="s">
+        <v>14</v>
+      </c>
+      <c r="J21" t="s">
+        <v>27</v>
+      </c>
+      <c r="K21" t="s">
+        <v>129</v>
+      </c>
+      <c r="M21" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>58</v>
-      </c>
-      <c r="B21">
-        <v>20</v>
-      </c>
-      <c r="C21">
-        <v>1</v>
-      </c>
-      <c r="D21" t="s">
-        <v>13</v>
-      </c>
-      <c r="I21" t="s">
-        <v>14</v>
-      </c>
-      <c r="J21" t="s">
-        <v>15</v>
-      </c>
-      <c r="K21" t="s">
-        <v>145</v>
-      </c>
-      <c r="M21" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="B22">
+        <v>6</v>
+      </c>
+      <c r="C22">
         <v>21</v>
       </c>
-      <c r="C22">
-        <v>11</v>
-      </c>
       <c r="D22" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="I22" t="s">
         <v>65</v>
       </c>
       <c r="J22" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="K22" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="M22" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>84</v>
       </c>
       <c r="B23">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="C23">
         <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>42</v>
+        <v>77</v>
       </c>
       <c r="I23" t="s">
-        <v>14</v>
+        <v>65</v>
       </c>
       <c r="J23" t="s">
         <v>27</v>
       </c>
       <c r="K23" t="s">
+        <v>155</v>
+      </c>
+      <c r="M23" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24">
+        <v>22</v>
+      </c>
+      <c r="C24">
+        <v>23</v>
+      </c>
+      <c r="D24" t="s">
+        <v>42</v>
+      </c>
+      <c r="I24" t="s">
+        <v>14</v>
+      </c>
+      <c r="J24" t="s">
+        <v>27</v>
+      </c>
+      <c r="K24" t="s">
         <v>147</v>
       </c>
-      <c r="M23" t="s">
+      <c r="M24" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>55</v>
-      </c>
-      <c r="B24">
-        <v>23</v>
-      </c>
-      <c r="C24">
-        <v>29</v>
-      </c>
-      <c r="D24" t="s">
-        <v>71</v>
-      </c>
-      <c r="I24" t="s">
-        <v>14</v>
-      </c>
-      <c r="J24" t="s">
-        <v>15</v>
-      </c>
-      <c r="K24" t="s">
-        <v>148</v>
-      </c>
-      <c r="M24" t="s">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25">
+        <v>25</v>
+      </c>
+      <c r="C25">
+        <v>24</v>
+      </c>
+      <c r="D25" t="s">
+        <v>46</v>
+      </c>
+      <c r="I25" t="s">
+        <v>14</v>
+      </c>
+      <c r="J25" t="s">
+        <v>27</v>
+      </c>
+      <c r="K25" t="s">
+        <v>150</v>
+      </c>
+      <c r="M25" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>78</v>
-      </c>
-      <c r="B25">
-        <v>24</v>
-      </c>
-      <c r="C25">
-        <v>8</v>
-      </c>
-      <c r="D25" t="s">
-        <v>72</v>
-      </c>
-      <c r="I25" t="s">
-        <v>65</v>
-      </c>
-      <c r="J25" t="s">
-        <v>24</v>
-      </c>
-      <c r="K25" t="s">
-        <v>149</v>
-      </c>
-      <c r="M25" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="B26">
+        <v>34</v>
+      </c>
+      <c r="C26">
         <v>25</v>
       </c>
-      <c r="C26">
-        <v>23</v>
-      </c>
       <c r="D26" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="I26" t="s">
         <v>14</v>
@@ -2077,180 +2086,180 @@
         <v>27</v>
       </c>
       <c r="K26" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="M26" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27">
+        <v>12</v>
+      </c>
+      <c r="C27">
+        <v>26</v>
+      </c>
+      <c r="D27" t="s">
+        <v>48</v>
+      </c>
+      <c r="I27" t="s">
+        <v>14</v>
+      </c>
+      <c r="J27" t="s">
+        <v>24</v>
+      </c>
+      <c r="K27" t="s">
+        <v>137</v>
+      </c>
+      <c r="M27" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>45</v>
+      </c>
+      <c r="B28">
+        <v>18</v>
+      </c>
+      <c r="C28">
+        <v>27</v>
+      </c>
+      <c r="D28" t="s">
+        <v>50</v>
+      </c>
+      <c r="I28" t="s">
+        <v>14</v>
+      </c>
+      <c r="J28" t="s">
+        <v>36</v>
+      </c>
+      <c r="K28" t="s">
+        <v>143</v>
+      </c>
+      <c r="M28" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>51</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29">
+        <v>28</v>
+      </c>
+      <c r="D29" t="s">
+        <v>52</v>
+      </c>
+      <c r="I29" t="s">
+        <v>14</v>
+      </c>
+      <c r="J29" t="s">
+        <v>27</v>
+      </c>
+      <c r="K29" t="s">
+        <v>126</v>
+      </c>
+      <c r="M29" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30">
+        <v>2</v>
+      </c>
+      <c r="C30">
+        <v>29</v>
+      </c>
+      <c r="D30" t="s">
+        <v>54</v>
+      </c>
+      <c r="I30" t="s">
+        <v>14</v>
+      </c>
+      <c r="J30" t="s">
+        <v>27</v>
+      </c>
+      <c r="K30" t="s">
+        <v>127</v>
+      </c>
+      <c r="M30" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>55</v>
+      </c>
+      <c r="B31">
+        <v>23</v>
+      </c>
+      <c r="C31">
+        <v>30</v>
+      </c>
+      <c r="D31" t="s">
+        <v>71</v>
+      </c>
+      <c r="I31" t="s">
+        <v>14</v>
+      </c>
+      <c r="J31" t="s">
+        <v>15</v>
+      </c>
+      <c r="K31" t="s">
+        <v>148</v>
+      </c>
+      <c r="M31" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
         <v>80</v>
       </c>
-      <c r="B27">
+      <c r="B32">
         <v>26</v>
       </c>
-      <c r="C27">
-        <v>30</v>
-      </c>
-      <c r="D27" t="s">
+      <c r="C32">
+        <v>31</v>
+      </c>
+      <c r="D32" t="s">
         <v>74</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I32" t="s">
         <v>65</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J32" t="s">
         <v>15</v>
       </c>
-      <c r="K27" t="s">
+      <c r="K32" t="s">
         <v>151</v>
       </c>
-      <c r="M27" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>81</v>
-      </c>
-      <c r="B28">
-        <v>27</v>
-      </c>
-      <c r="C28">
-        <v>18</v>
-      </c>
-      <c r="D28" t="s">
-        <v>73</v>
-      </c>
-      <c r="I28" t="s">
-        <v>65</v>
-      </c>
-      <c r="J28" t="s">
-        <v>24</v>
-      </c>
-      <c r="K28" t="s">
-        <v>152</v>
-      </c>
-      <c r="M28" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>82</v>
-      </c>
-      <c r="B29">
-        <v>28</v>
-      </c>
-      <c r="C29">
-        <v>34</v>
-      </c>
-      <c r="D29" t="s">
-        <v>61</v>
-      </c>
-      <c r="I29" t="s">
-        <v>14</v>
-      </c>
-      <c r="J29" t="s">
-        <v>57</v>
-      </c>
-      <c r="K29" t="s">
-        <v>153</v>
-      </c>
-      <c r="M29" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="M32" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
         <v>83</v>
       </c>
-      <c r="B30">
+      <c r="B33">
         <v>29</v>
       </c>
-      <c r="C30">
-        <v>31</v>
-      </c>
-      <c r="D30" t="s">
+      <c r="C33">
+        <v>32</v>
+      </c>
+      <c r="D33" t="s">
         <v>75</v>
-      </c>
-      <c r="I30" t="s">
-        <v>65</v>
-      </c>
-      <c r="J30" t="s">
-        <v>15</v>
-      </c>
-      <c r="K30" t="s">
-        <v>154</v>
-      </c>
-      <c r="M30" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>84</v>
-      </c>
-      <c r="B31">
-        <v>30</v>
-      </c>
-      <c r="C31">
-        <v>21</v>
-      </c>
-      <c r="D31" t="s">
-        <v>77</v>
-      </c>
-      <c r="I31" t="s">
-        <v>65</v>
-      </c>
-      <c r="J31" t="s">
-        <v>27</v>
-      </c>
-      <c r="K31" t="s">
-        <v>155</v>
-      </c>
-      <c r="M31" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>85</v>
-      </c>
-      <c r="B32">
-        <v>31</v>
-      </c>
-      <c r="C32">
-        <v>33</v>
-      </c>
-      <c r="D32" t="s">
-        <v>59</v>
-      </c>
-      <c r="I32" t="s">
-        <v>14</v>
-      </c>
-      <c r="J32" t="s">
-        <v>57</v>
-      </c>
-      <c r="K32" t="s">
-        <v>156</v>
-      </c>
-      <c r="M32" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>86</v>
-      </c>
-      <c r="B33">
-        <v>32</v>
-      </c>
-      <c r="C33">
-        <v>2</v>
-      </c>
-      <c r="D33" t="s">
-        <v>76</v>
       </c>
       <c r="I33" t="s">
         <v>65</v>
@@ -2259,24 +2268,24 @@
         <v>15</v>
       </c>
       <c r="K33" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="M33" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B34">
+        <v>35</v>
+      </c>
+      <c r="C34">
         <v>33</v>
       </c>
-      <c r="C34">
-        <v>35</v>
-      </c>
       <c r="D34" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="I34" t="s">
         <v>14</v>
@@ -2285,50 +2294,50 @@
         <v>57</v>
       </c>
       <c r="K34" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="M34" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>85</v>
+      </c>
+      <c r="B35">
+        <v>31</v>
+      </c>
+      <c r="C35">
+        <v>34</v>
+      </c>
+      <c r="D35" t="s">
+        <v>59</v>
+      </c>
+      <c r="I35" t="s">
+        <v>14</v>
+      </c>
+      <c r="J35" t="s">
+        <v>57</v>
+      </c>
+      <c r="K35" t="s">
+        <v>156</v>
+      </c>
+      <c r="M35" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>88</v>
-      </c>
-      <c r="B35">
-        <v>34</v>
-      </c>
-      <c r="C35">
-        <v>24</v>
-      </c>
-      <c r="D35" t="s">
-        <v>44</v>
-      </c>
-      <c r="I35" t="s">
-        <v>14</v>
-      </c>
-      <c r="J35" t="s">
-        <v>27</v>
-      </c>
-      <c r="K35" t="s">
-        <v>159</v>
-      </c>
-      <c r="M35" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="B36">
+        <v>28</v>
+      </c>
+      <c r="C36">
         <v>35</v>
       </c>
-      <c r="C36">
-        <v>32</v>
-      </c>
       <c r="D36" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="I36" t="s">
         <v>14</v>
@@ -2337,22 +2346,49 @@
         <v>57</v>
       </c>
       <c r="K36" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="M36" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>87</v>
+      </c>
+      <c r="B37">
+        <v>33</v>
+      </c>
+      <c r="C37">
+        <v>36</v>
+      </c>
+      <c r="D37" t="s">
+        <v>63</v>
+      </c>
+      <c r="I37" t="s">
+        <v>14</v>
+      </c>
+      <c r="J37" t="s">
+        <v>57</v>
+      </c>
+      <c r="K37" t="s">
+        <v>158</v>
+      </c>
+      <c r="M37" t="s">
         <v>125</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L36" xr:uid="{0D7D8C5C-82D0-4767-86A0-EC7D017C2964}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L36">
-      <sortCondition ref="B1:B36"/>
+  <autoFilter ref="A1:L37" xr:uid="{0D7D8C5C-82D0-4767-86A0-EC7D017C2964}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:L38">
+      <sortCondition ref="C1:C37"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="18" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="M6" r:id="rId1" xr:uid="{9D13AB1B-17E5-47B8-8BB4-A42EF0F05C18}"/>
-    <hyperlink ref="M13" r:id="rId2" xr:uid="{5D408525-0FF4-4DD4-8542-509FE990F36A}"/>
+    <hyperlink ref="M14" r:id="rId2" xr:uid="{5D408525-0FF4-4DD4-8542-509FE990F36A}"/>
+    <hyperlink ref="K8" r:id="rId3" xr:uid="{DF43A1D2-992A-48FE-A6AB-44640F3E59CD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Hyrule Warriors Timeline Fix
</commit_message>
<xml_diff>
--- a/ZELDA.xlsx
+++ b/ZELDA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAB5AA8B-AA15-48EC-A67F-49733D5729A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D60549A5-EBFE-4C41-AF98-D3CC283F1008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{544A5710-79AF-4C5F-8C3A-ADA1AE421E72}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="165">
   <si>
     <t>id</t>
   </si>
@@ -515,6 +515,9 @@
   </si>
   <si>
     <t>https://www.igdb.com/games/the-legend-of-zelda-ocarina-of-time--1</t>
+  </si>
+  <si>
+    <t>Non-Canon Spinoff</t>
   </si>
 </sst>
 </file>
@@ -1849,7 +1852,7 @@
         <v>67</v>
       </c>
       <c r="J17" t="s">
-        <v>24</v>
+        <v>164</v>
       </c>
       <c r="K17" t="s">
         <v>139</v>
@@ -2213,7 +2216,7 @@
         <v>14</v>
       </c>
       <c r="J31" t="s">
-        <v>15</v>
+        <v>164</v>
       </c>
       <c r="K31" t="s">
         <v>148</v>
@@ -2239,7 +2242,7 @@
         <v>65</v>
       </c>
       <c r="J32" t="s">
-        <v>15</v>
+        <v>164</v>
       </c>
       <c r="K32" t="s">
         <v>151</v>
@@ -2265,7 +2268,7 @@
         <v>65</v>
       </c>
       <c r="J33" t="s">
-        <v>15</v>
+        <v>164</v>
       </c>
       <c r="K33" t="s">
         <v>154</v>
@@ -2317,7 +2320,7 @@
         <v>14</v>
       </c>
       <c r="J35" t="s">
-        <v>57</v>
+        <v>164</v>
       </c>
       <c r="K35" t="s">
         <v>156</v>

</xml_diff>

<commit_message>
Zelda Canon States Fix
</commit_message>
<xml_diff>
--- a/ZELDA.xlsx
+++ b/ZELDA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\timeline-site\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D60549A5-EBFE-4C41-AF98-D3CC283F1008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B1DB79-8C6B-4EC9-BAA0-F249DB438458}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{544A5710-79AF-4C5F-8C3A-ADA1AE421E72}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="167">
   <si>
     <t>id</t>
   </si>
@@ -67,9 +67,6 @@
     <t>The Legend of Zelda: Skyward Sword</t>
   </si>
   <si>
-    <t>Video Game</t>
-  </si>
-  <si>
     <t>Adult Timeline, Child Timeline, Downfall Timeline</t>
   </si>
   <si>
@@ -220,15 +217,9 @@
     <t>The Legend of Zelda: Link's Awakening DX</t>
   </si>
   <si>
-    <t>Video Game (Remaster)</t>
-  </si>
-  <si>
     <t>Freshly-Picked Tingle's Rosy Rupeeland</t>
   </si>
   <si>
-    <t>Video Game (Spinoff)</t>
-  </si>
-  <si>
     <t>Link's Crossbow Training</t>
   </si>
   <si>
@@ -518,6 +509,21 @@
   </si>
   <si>
     <t>Non-Canon Spinoff</t>
+  </si>
+  <si>
+    <t>Video Game (3D)</t>
+  </si>
+  <si>
+    <t>Video Game (3D Remaster)</t>
+  </si>
+  <si>
+    <t>Video Game (2D)</t>
+  </si>
+  <si>
+    <t>Video Game (2D/3D Blend)</t>
+  </si>
+  <si>
+    <t>Video Game (2D Remaster)</t>
   </si>
 </sst>
 </file>
@@ -1442,12 +1448,12 @@
         <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B2">
         <v>20</v>
@@ -1459,21 +1465,21 @@
         <v>13</v>
       </c>
       <c r="I2" t="s">
+        <v>162</v>
+      </c>
+      <c r="J2" t="s">
         <v>14</v>
       </c>
-      <c r="J2" t="s">
-        <v>15</v>
-      </c>
       <c r="K2" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="M2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B3">
         <v>32</v>
@@ -1482,24 +1488,24 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="I3" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="J3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K3" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="M3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4">
         <v>13</v>
@@ -1508,24 +1514,24 @@
         <v>3</v>
       </c>
       <c r="D4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I4" t="s">
+        <v>164</v>
+      </c>
+      <c r="J4" t="s">
         <v>14</v>
       </c>
-      <c r="J4" t="s">
-        <v>15</v>
-      </c>
       <c r="K4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="M4" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5">
         <v>10</v>
@@ -1534,24 +1540,24 @@
         <v>4</v>
       </c>
       <c r="D5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I5" t="s">
+        <v>164</v>
+      </c>
+      <c r="J5" t="s">
         <v>14</v>
       </c>
-      <c r="J5" t="s">
-        <v>15</v>
-      </c>
       <c r="K5" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="M5" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B6">
         <v>5</v>
@@ -1560,24 +1566,24 @@
         <v>5</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I6" t="s">
+        <v>162</v>
+      </c>
+      <c r="J6" t="s">
         <v>14</v>
       </c>
-      <c r="J6" t="s">
-        <v>15</v>
-      </c>
       <c r="K6" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B7">
         <v>19</v>
@@ -1586,24 +1592,24 @@
         <v>6</v>
       </c>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="I7" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="J7" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K7" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="M7" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="B8">
         <v>36</v>
@@ -1612,24 +1618,24 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="I8" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="J8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="M8" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9">
         <v>7</v>
@@ -1638,24 +1644,24 @@
         <v>8</v>
       </c>
       <c r="D9" t="s">
+        <v>22</v>
+      </c>
+      <c r="I9" t="s">
+        <v>162</v>
+      </c>
+      <c r="J9" t="s">
         <v>23</v>
       </c>
-      <c r="I9" t="s">
-        <v>14</v>
-      </c>
-      <c r="J9" t="s">
-        <v>24</v>
-      </c>
       <c r="K9" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="M9" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B10">
         <v>24</v>
@@ -1664,24 +1670,24 @@
         <v>9</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="I10" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="J10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K10" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="M10" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11">
         <v>3</v>
@@ -1690,24 +1696,24 @@
         <v>10</v>
       </c>
       <c r="D11" t="s">
+        <v>25</v>
+      </c>
+      <c r="I11" t="s">
+        <v>164</v>
+      </c>
+      <c r="J11" t="s">
         <v>26</v>
       </c>
-      <c r="I11" t="s">
-        <v>14</v>
-      </c>
-      <c r="J11" t="s">
-        <v>27</v>
-      </c>
       <c r="K11" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="M11" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B12">
         <v>11</v>
@@ -1716,24 +1722,24 @@
         <v>11</v>
       </c>
       <c r="D12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I12" t="s">
-        <v>14</v>
+        <v>162</v>
       </c>
       <c r="J12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K12" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="M12" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B13">
         <v>21</v>
@@ -1742,24 +1748,24 @@
         <v>12</v>
       </c>
       <c r="D13" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="I13" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="J13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K13" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="M13" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B14">
         <v>8</v>
@@ -1768,24 +1774,24 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="I14" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="J14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K14" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15">
         <v>9</v>
@@ -1794,19 +1800,19 @@
         <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I15" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="J15" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K15" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="M15" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.45">
@@ -1820,24 +1826,24 @@
         <v>15</v>
       </c>
       <c r="D16" t="s">
+        <v>34</v>
+      </c>
+      <c r="I16" t="s">
+        <v>165</v>
+      </c>
+      <c r="J16" t="s">
         <v>35</v>
       </c>
-      <c r="I16" t="s">
-        <v>14</v>
-      </c>
-      <c r="J16" t="s">
-        <v>36</v>
-      </c>
       <c r="K16" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="M16" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B17">
         <v>14</v>
@@ -1846,24 +1852,24 @@
         <v>16</v>
       </c>
       <c r="D17" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I17" t="s">
-        <v>67</v>
+        <v>164</v>
       </c>
       <c r="J17" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K17" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="M17" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18">
         <v>17</v>
@@ -1872,24 +1878,24 @@
         <v>17</v>
       </c>
       <c r="D18" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I18" t="s">
-        <v>67</v>
+        <v>162</v>
       </c>
       <c r="J18" t="s">
-        <v>24</v>
+        <v>161</v>
       </c>
       <c r="K18" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="M18" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B19">
         <v>15</v>
@@ -1898,24 +1904,24 @@
         <v>18</v>
       </c>
       <c r="D19" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="I19" t="s">
-        <v>14</v>
+        <v>162</v>
       </c>
       <c r="J19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K19" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="M19" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B20">
         <v>27</v>
@@ -1924,24 +1930,24 @@
         <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="I20" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="J20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K20" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="M20" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B21">
         <v>4</v>
@@ -1950,24 +1956,24 @@
         <v>20</v>
       </c>
       <c r="D21" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="I21" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="J21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K21" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="M21" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B22">
         <v>6</v>
@@ -1976,24 +1982,24 @@
         <v>21</v>
       </c>
       <c r="D22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I22" t="s">
-        <v>65</v>
+        <v>166</v>
       </c>
       <c r="J22" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K22" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="M22" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B23">
         <v>30</v>
@@ -2002,24 +2008,24 @@
         <v>22</v>
       </c>
       <c r="D23" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I23" t="s">
-        <v>65</v>
+        <v>166</v>
       </c>
       <c r="J23" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K23" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="M23" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B24">
         <v>22</v>
@@ -2028,24 +2034,24 @@
         <v>23</v>
       </c>
       <c r="D24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="I24" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="J24" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K24" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="M24" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B25">
         <v>25</v>
@@ -2054,24 +2060,24 @@
         <v>24</v>
       </c>
       <c r="D25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I25" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="J25" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K25" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="M25" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B26">
         <v>34</v>
@@ -2080,24 +2086,24 @@
         <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="I26" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="J26" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K26" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="M26" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B27">
         <v>12</v>
@@ -2106,24 +2112,24 @@
         <v>26</v>
       </c>
       <c r="D27" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="I27" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="J27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="K27" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="M27" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B28">
         <v>18</v>
@@ -2132,24 +2138,24 @@
         <v>27</v>
       </c>
       <c r="D28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I28" t="s">
-        <v>14</v>
+        <v>165</v>
       </c>
       <c r="J28" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K28" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="M28" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B29">
         <v>1</v>
@@ -2158,24 +2164,24 @@
         <v>28</v>
       </c>
       <c r="D29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I29" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="J29" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K29" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="M29" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B30">
         <v>2</v>
@@ -2184,24 +2190,24 @@
         <v>29</v>
       </c>
       <c r="D30" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I30" t="s">
-        <v>14</v>
+        <v>164</v>
       </c>
       <c r="J30" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="K30" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="M30" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B31">
         <v>23</v>
@@ -2210,24 +2216,24 @@
         <v>30</v>
       </c>
       <c r="D31" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I31" t="s">
-        <v>14</v>
+        <v>162</v>
       </c>
       <c r="J31" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K31" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="M31" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B32">
         <v>26</v>
@@ -2236,24 +2242,24 @@
         <v>31</v>
       </c>
       <c r="D32" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="I32" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="J32" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K32" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="M32" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B33">
         <v>29</v>
@@ -2262,24 +2268,24 @@
         <v>32</v>
       </c>
       <c r="D33" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I33" t="s">
-        <v>65</v>
+        <v>163</v>
       </c>
       <c r="J33" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K33" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="M33" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B34">
         <v>35</v>
@@ -2288,24 +2294,24 @@
         <v>33</v>
       </c>
       <c r="D34" t="s">
+        <v>55</v>
+      </c>
+      <c r="I34" t="s">
+        <v>162</v>
+      </c>
+      <c r="J34" t="s">
         <v>56</v>
       </c>
-      <c r="I34" t="s">
-        <v>14</v>
-      </c>
-      <c r="J34" t="s">
-        <v>57</v>
-      </c>
       <c r="K34" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="M34" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B35">
         <v>31</v>
@@ -2314,24 +2320,24 @@
         <v>34</v>
       </c>
       <c r="D35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I35" t="s">
-        <v>14</v>
+        <v>162</v>
       </c>
       <c r="J35" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K35" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="M35" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B36">
         <v>28</v>
@@ -2340,24 +2346,24 @@
         <v>35</v>
       </c>
       <c r="D36" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I36" t="s">
-        <v>14</v>
+        <v>162</v>
       </c>
       <c r="J36" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K36" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="M36" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B37">
         <v>33</v>
@@ -2366,19 +2372,19 @@
         <v>36</v>
       </c>
       <c r="D37" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="I37" t="s">
-        <v>14</v>
+        <v>162</v>
       </c>
       <c r="J37" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="K37" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="M37" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>